<commit_message>
add MEX, ARG, CRI in sel
</commit_message>
<xml_diff>
--- a/input_data/sna_country_data/URY/cei.xlsx
+++ b/input_data/sna_country_data/URY/cei.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42476" uniqueCount="24329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43050" uniqueCount="24329">
   <si>
     <t>code</t>
   </si>
@@ -73781,7 +73781,7 @@
         <v>25446.753598644849</v>
       </c>
       <c r="H34" s="1">
-        <v>25446.753598644718</v>
+        <v>25446.753598644849</v>
       </c>
     </row>
     <row r="35">
@@ -73807,24 +73807,22 @@
         <v>25446.753598644718</v>
       </c>
       <c r="H35" s="1">
-        <v>25446.753598644849</v>
+        <v>25446.753598644718</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>24286</v>
+        <v>24284</v>
       </c>
       <c r="B36" t="s">
-        <v>24322</v>
+        <v>24320</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>79482.446760280014</v>
-      </c>
-      <c r="F36" s="1">
-        <v>79482.446760280014</v>
-      </c>
+        <v>926.5806651800001</v>
+      </c>
+      <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
     </row>
@@ -73848,17 +73846,19 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24284</v>
+        <v>24286</v>
       </c>
       <c r="B38" t="s">
-        <v>24320</v>
+        <v>24322</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>926.5806651800001</v>
-      </c>
-      <c r="F38" s="1"/>
+        <v>79482.446760280014</v>
+      </c>
+      <c r="F38" s="1">
+        <v>79482.446760280014</v>
+      </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
@@ -74443,10 +74443,10 @@
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1">
+        <v>-10570.43407502865</v>
+      </c>
+      <c r="F27" s="1">
         <v>-10570.434075028639</v>
-      </c>
-      <c r="F27" s="1">
-        <v>-10570.43407502865</v>
       </c>
       <c r="G27" s="1">
         <v>124508.5573505638</v>
@@ -74523,10 +74523,10 @@
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1">
+        <v>-10570.434075028639</v>
+      </c>
+      <c r="F31" s="1">
         <v>-10570.43407502865</v>
-      </c>
-      <c r="F31" s="1">
-        <v>-10570.434075028639</v>
       </c>
       <c r="G31" s="1">
         <v>124508.5573505638</v>
@@ -74593,16 +74593,16 @@
         <v>-14574.434848447811</v>
       </c>
       <c r="E34" s="1">
+        <v>-66950.582658753861</v>
+      </c>
+      <c r="F34" s="1">
         <v>-66950.582658753847</v>
       </c>
-      <c r="F34" s="1">
-        <v>-66950.582658753861</v>
-      </c>
       <c r="G34" s="1">
-        <v>55330.055140544697</v>
+        <v>55330.055140544151</v>
       </c>
       <c r="H34" s="1">
-        <v>55330.055140544697</v>
+        <v>55330.055140544151</v>
       </c>
     </row>
     <row r="35">
@@ -74619,37 +74619,35 @@
         <v>-14574.43484844782</v>
       </c>
       <c r="E35" s="1">
+        <v>-66950.582658753847</v>
+      </c>
+      <c r="F35" s="1">
         <v>-66950.582658753861</v>
       </c>
-      <c r="F35" s="1">
-        <v>-66950.582658753847</v>
-      </c>
       <c r="G35" s="1">
-        <v>55330.055140544151</v>
+        <v>55330.055140544697</v>
       </c>
       <c r="H35" s="1">
-        <v>55330.055140544151</v>
+        <v>55330.055140544697</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>24285</v>
+        <v>24286</v>
       </c>
       <c r="B36" t="s">
-        <v>24321</v>
+        <v>24322</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>181558.9914336357</v>
-      </c>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1">
-        <v>310.92989817709997</v>
-      </c>
-      <c r="H36" s="1">
-        <v>223683.25268700649</v>
-      </c>
+        <v>147042.35994689999</v>
+      </c>
+      <c r="F36" s="1">
+        <v>147042.21094677999</v>
+      </c>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" t="s">
@@ -74669,21 +74667,23 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24286</v>
+        <v>24285</v>
       </c>
       <c r="B38" t="s">
-        <v>24322</v>
+        <v>24321</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>147042.35994689999</v>
-      </c>
-      <c r="F38" s="1">
-        <v>147042.21094677999</v>
-      </c>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
+        <v>181558.9914336357</v>
+      </c>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1">
+        <v>310.92989817709997</v>
+      </c>
+      <c r="H38" s="1">
+        <v>223683.25268700649</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>
@@ -75271,7 +75271,7 @@
         <v>-25017.388782343201</v>
       </c>
       <c r="F27" s="1">
-        <v>-25017.38878234318</v>
+        <v>-25017.388782343201</v>
       </c>
       <c r="G27" s="1">
         <v>118456.4656790759</v>
@@ -75351,7 +75351,7 @@
         <v>-25017.38878234318</v>
       </c>
       <c r="F31" s="1">
-        <v>-25017.388782343201</v>
+        <v>-25017.38878234318</v>
       </c>
       <c r="G31" s="1">
         <v>118456.4656790759</v>
@@ -75421,13 +75421,13 @@
         <v>-63565.770979082881</v>
       </c>
       <c r="F34" s="1">
-        <v>-63565.770979082881</v>
+        <v>-63565.818181042087</v>
       </c>
       <c r="G34" s="1">
         <v>43782.161676835007</v>
       </c>
       <c r="H34" s="1">
-        <v>43782.161676835007</v>
+        <v>43782.161676834643</v>
       </c>
     </row>
     <row r="35">
@@ -75447,52 +75447,52 @@
         <v>-63565.818181042087</v>
       </c>
       <c r="F35" s="1">
-        <v>-63565.818181042087</v>
+        <v>-63565.770979082881</v>
       </c>
       <c r="G35" s="1">
         <v>43782.161676834643</v>
       </c>
       <c r="H35" s="1">
-        <v>43782.161676834643</v>
+        <v>43782.161676835007</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>24286</v>
+        <v>24285</v>
       </c>
       <c r="B36" t="s">
-        <v>24322</v>
+        <v>24321</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>170013.75605207999</v>
-      </c>
-      <c r="F36" s="1">
-        <v>170013.75605207999</v>
-      </c>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
+        <v>201604.21968480741</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1">
+        <v>337.34758922499998</v>
+      </c>
+      <c r="H36" s="1">
+        <v>253381.7166756459</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24285</v>
+        <v>24286</v>
       </c>
       <c r="B37" t="s">
-        <v>24321</v>
+        <v>24322</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>201604.21968480741</v>
-      </c>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1">
-        <v>337.34758922499998</v>
-      </c>
-      <c r="H37" s="1">
-        <v>253381.7166756459</v>
-      </c>
+        <v>170013.75605207999</v>
+      </c>
+      <c r="F37" s="1">
+        <v>170013.75605207999</v>
+      </c>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
@@ -76234,13 +76234,13 @@
         <v>5442.5976345336867</v>
       </c>
       <c r="D34" s="1">
-        <v>5442.5976345336967</v>
+        <v>5442.5976345336867</v>
       </c>
       <c r="E34" s="1">
+        <v>-49773.892247343349</v>
+      </c>
+      <c r="F34" s="1">
         <v>-49773.892247342999</v>
-      </c>
-      <c r="F34" s="1">
-        <v>-49773.892247343349</v>
       </c>
       <c r="G34" s="1">
         <v>33283.712597372418</v>
@@ -76260,13 +76260,13 @@
         <v>5442.5976345336967</v>
       </c>
       <c r="D35" s="1">
-        <v>5442.5976345336867</v>
+        <v>5442.5976345336967</v>
       </c>
       <c r="E35" s="1">
+        <v>-49773.892247342999</v>
+      </c>
+      <c r="F35" s="1">
         <v>-49773.892247343349</v>
-      </c>
-      <c r="F35" s="1">
-        <v>-49773.892247342999</v>
       </c>
       <c r="G35" s="1">
         <v>33283.712597372112</v>
@@ -76297,35 +76297,35 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24286</v>
+        <v>24284</v>
       </c>
       <c r="B37" t="s">
-        <v>24322</v>
+        <v>24320</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>207169.67690947151</v>
-      </c>
-      <c r="F37" s="1">
-        <v>207169.67690947151</v>
-      </c>
+        <v>1640.019891895929</v>
+      </c>
+      <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24284</v>
+        <v>24286</v>
       </c>
       <c r="B38" t="s">
-        <v>24320</v>
+        <v>24322</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>1640.019891895929</v>
-      </c>
-      <c r="F38" s="1"/>
+        <v>207169.67690947151</v>
+      </c>
+      <c r="F38" s="1">
+        <v>207169.67690947151</v>
+      </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
@@ -76913,7 +76913,7 @@
         <v>-47487.012322160823</v>
       </c>
       <c r="F27" s="1">
-        <v>-47487.012322160852</v>
+        <v>-47487.012322160823</v>
       </c>
       <c r="G27" s="1">
         <v>137422.3722114753</v>
@@ -76991,7 +76991,7 @@
         <v>-47487.012322160852</v>
       </c>
       <c r="F31" s="1">
-        <v>-47487.012322160823</v>
+        <v>-47487.012322160852</v>
       </c>
       <c r="G31" s="1">
         <v>137422.3722114753</v>
@@ -77061,7 +77061,7 @@
         <v>-63947.039175029808</v>
       </c>
       <c r="F34" s="1">
-        <v>-63947.039175029808</v>
+        <v>-63947.039175030113</v>
       </c>
       <c r="G34" s="1">
         <v>39248.472782472993</v>
@@ -77087,7 +77087,7 @@
         <v>-63947.039175030113</v>
       </c>
       <c r="F35" s="1">
-        <v>-63947.039175030113</v>
+        <v>-63947.039175029808</v>
       </c>
       <c r="G35" s="1">
         <v>39248.472782472847</v>
@@ -77114,41 +77114,41 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24286</v>
+        <v>24285</v>
       </c>
       <c r="B37" t="s">
-        <v>24322</v>
+        <v>24321</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>200663.39336498949</v>
-      </c>
-      <c r="F37" s="1">
-        <v>200663.39336498949</v>
-      </c>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
+        <v>239376.743428952</v>
+      </c>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1">
+        <v>402.67289956090139</v>
+      </c>
+      <c r="H37" s="1">
+        <v>298520.24294644757</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24285</v>
+        <v>24286</v>
       </c>
       <c r="B38" t="s">
-        <v>24321</v>
+        <v>24322</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>239376.743428952</v>
-      </c>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1">
-        <v>402.67289956090139</v>
-      </c>
-      <c r="H38" s="1">
-        <v>298520.24294644757</v>
-      </c>
+        <v>200663.39336498949</v>
+      </c>
+      <c r="F38" s="1">
+        <v>200663.39336498949</v>
+      </c>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
     </row>
   </sheetData>
 </worksheet>
@@ -77872,7 +77872,7 @@
         <v>10171.468589380889</v>
       </c>
       <c r="D34" s="1">
-        <v>10171.459058987501</v>
+        <v>10171.468589380889</v>
       </c>
       <c r="E34" s="1">
         <v>-79545.106801385089</v>
@@ -77898,7 +77898,7 @@
         <v>10171.459058987501</v>
       </c>
       <c r="D35" s="1">
-        <v>10171.468589380889</v>
+        <v>10171.459058987501</v>
       </c>
       <c r="E35" s="1">
         <v>-79545.106801385089</v>
@@ -77935,35 +77935,35 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24286</v>
+        <v>24284</v>
       </c>
       <c r="B37" t="s">
-        <v>24322</v>
+        <v>24320</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>242248.42014405999</v>
-      </c>
-      <c r="F37" s="1">
-        <v>242248.42014405999</v>
-      </c>
+        <v>1625.492093275358</v>
+      </c>
+      <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24284</v>
+        <v>24286</v>
       </c>
       <c r="B38" t="s">
-        <v>24320</v>
+        <v>24322</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>1625.492093275358</v>
-      </c>
-      <c r="F38" s="1"/>
+        <v>242248.42014405999</v>
+      </c>
+      <c r="F38" s="1">
+        <v>242248.42014405999</v>
+      </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
@@ -78546,7 +78546,7 @@
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1">
-        <v>-25100.98923128075</v>
+        <v>-25100.989231280721</v>
       </c>
       <c r="F27" s="1">
         <v>-25100.98923128075</v>
@@ -78624,7 +78624,7 @@
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1">
-        <v>-25100.989231280721</v>
+        <v>-25100.98923128075</v>
       </c>
       <c r="F31" s="1">
         <v>-25100.989231280721</v>
@@ -78700,10 +78700,10 @@
         <v>-60032.164387225363</v>
       </c>
       <c r="G34" s="1">
+        <v>50492.474199901873</v>
+      </c>
+      <c r="H34" s="1">
         <v>50492.474199902237</v>
-      </c>
-      <c r="H34" s="1">
-        <v>50492.474199901873</v>
       </c>
     </row>
     <row r="35">
@@ -78726,10 +78726,10 @@
         <v>-60032.164387225363</v>
       </c>
       <c r="G35" s="1">
+        <v>50492.474199902237</v>
+      </c>
+      <c r="H35" s="1">
         <v>50492.474199901873</v>
-      </c>
-      <c r="H35" s="1">
-        <v>50492.474199902237</v>
       </c>
     </row>
     <row r="36">
@@ -78750,41 +78750,41 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24286</v>
+        <v>24285</v>
       </c>
       <c r="B37" t="s">
-        <v>24322</v>
+        <v>24321</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>264574.52162751998</v>
-      </c>
-      <c r="F37" s="1">
-        <v>264574.52162751998</v>
-      </c>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
+        <v>272538.25067318691</v>
+      </c>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1">
+        <v>456.40441621169998</v>
+      </c>
+      <c r="H37" s="1">
+        <v>335741.85541967727</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24285</v>
+        <v>24286</v>
       </c>
       <c r="B38" t="s">
-        <v>24321</v>
+        <v>24322</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>272538.25067318691</v>
-      </c>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1">
-        <v>456.40441621169998</v>
-      </c>
-      <c r="H38" s="1">
-        <v>335741.85541967727</v>
-      </c>
+        <v>264574.52162751998</v>
+      </c>
+      <c r="F38" s="1">
+        <v>264574.52162751998</v>
+      </c>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
add 3 digit codes in SNA
</commit_message>
<xml_diff>
--- a/input_data/sna_country_data/URY/cei.xlsx
+++ b/input_data/sna_country_data/URY/cei.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43050" uniqueCount="24329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44772" uniqueCount="24329">
   <si>
     <t>code</t>
   </si>
@@ -73624,10 +73624,10 @@
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1">
-        <v>-3264.8749993161441</v>
+        <v>-3264.8749993161591</v>
       </c>
       <c r="F27" s="1">
-        <v>-3264.8749993161441</v>
+        <v>-3264.8749993161591</v>
       </c>
       <c r="G27" s="1">
         <v>65128.014697722727</v>
@@ -73704,10 +73704,10 @@
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1">
-        <v>-3264.8749993161591</v>
+        <v>-3264.8749993161441</v>
       </c>
       <c r="F31" s="1">
-        <v>-3264.8749993161591</v>
+        <v>-3264.8749993161441</v>
       </c>
       <c r="G31" s="1">
         <v>65128.014697722727</v>
@@ -73781,7 +73781,7 @@
         <v>25446.753598644849</v>
       </c>
       <c r="H34" s="1">
-        <v>25446.753598644849</v>
+        <v>25446.753598644718</v>
       </c>
     </row>
     <row r="35">
@@ -73807,42 +73807,42 @@
         <v>25446.753598644718</v>
       </c>
       <c r="H35" s="1">
-        <v>25446.753598644718</v>
+        <v>25446.753598644849</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>24284</v>
+        <v>24285</v>
       </c>
       <c r="B36" t="s">
-        <v>24320</v>
+        <v>24321</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>926.5806651800001</v>
+        <v>113976.0975413</v>
       </c>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
+      <c r="H36" s="1">
+        <v>137582.86030768359</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24285</v>
+        <v>24284</v>
       </c>
       <c r="B37" t="s">
-        <v>24321</v>
+        <v>24320</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>113976.0975413</v>
+        <v>926.5806651800001</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
-      <c r="H37" s="1">
-        <v>137582.86030768359</v>
-      </c>
+      <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
@@ -74446,7 +74446,7 @@
         <v>-10570.43407502865</v>
       </c>
       <c r="F27" s="1">
-        <v>-10570.434075028639</v>
+        <v>-10570.43407502865</v>
       </c>
       <c r="G27" s="1">
         <v>124508.5573505638</v>
@@ -74526,7 +74526,7 @@
         <v>-10570.434075028639</v>
       </c>
       <c r="F31" s="1">
-        <v>-10570.43407502865</v>
+        <v>-10570.434075028639</v>
       </c>
       <c r="G31" s="1">
         <v>124508.5573505638</v>
@@ -74599,7 +74599,7 @@
         <v>-66950.582658753847</v>
       </c>
       <c r="G34" s="1">
-        <v>55330.055140544151</v>
+        <v>55330.055140544697</v>
       </c>
       <c r="H34" s="1">
         <v>55330.055140544151</v>
@@ -74625,7 +74625,7 @@
         <v>-66950.582658753861</v>
       </c>
       <c r="G35" s="1">
-        <v>55330.055140544697</v>
+        <v>55330.055140544151</v>
       </c>
       <c r="H35" s="1">
         <v>55330.055140544697</v>
@@ -74633,57 +74633,57 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>24286</v>
+        <v>24285</v>
       </c>
       <c r="B36" t="s">
-        <v>24322</v>
+        <v>24321</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>147042.35994689999</v>
-      </c>
-      <c r="F36" s="1">
-        <v>147042.21094677999</v>
-      </c>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
+        <v>181558.9914336357</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1">
+        <v>310.92989817709997</v>
+      </c>
+      <c r="H36" s="1">
+        <v>223683.25268700649</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24284</v>
+        <v>24286</v>
       </c>
       <c r="B37" t="s">
-        <v>24320</v>
+        <v>24322</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>1410.7265588499999</v>
-      </c>
-      <c r="F37" s="1"/>
+        <v>147042.35994689999</v>
+      </c>
+      <c r="F37" s="1">
+        <v>147042.21094677999</v>
+      </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24285</v>
+        <v>24284</v>
       </c>
       <c r="B38" t="s">
-        <v>24321</v>
+        <v>24320</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>181558.9914336357</v>
+        <v>1410.7265588499999</v>
       </c>
       <c r="F38" s="1"/>
-      <c r="G38" s="1">
-        <v>310.92989817709997</v>
-      </c>
-      <c r="H38" s="1">
-        <v>223683.25268700649</v>
-      </c>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
     </row>
   </sheetData>
 </worksheet>
@@ -75271,7 +75271,7 @@
         <v>-25017.388782343201</v>
       </c>
       <c r="F27" s="1">
-        <v>-25017.388782343201</v>
+        <v>-25017.38878234318</v>
       </c>
       <c r="G27" s="1">
         <v>118456.4656790759</v>
@@ -75351,7 +75351,7 @@
         <v>-25017.38878234318</v>
       </c>
       <c r="F31" s="1">
-        <v>-25017.38878234318</v>
+        <v>-25017.388782343201</v>
       </c>
       <c r="G31" s="1">
         <v>118456.4656790759</v>
@@ -75415,19 +75415,19 @@
         <v>-4009.0753441289771</v>
       </c>
       <c r="D34" s="1">
-        <v>-4009.0753441289771</v>
+        <v>-4009.0753441289712</v>
       </c>
       <c r="E34" s="1">
-        <v>-63565.770979082881</v>
+        <v>-63565.818181042087</v>
       </c>
       <c r="F34" s="1">
         <v>-63565.818181042087</v>
       </c>
       <c r="G34" s="1">
+        <v>43782.161676834643</v>
+      </c>
+      <c r="H34" s="1">
         <v>43782.161676835007</v>
-      </c>
-      <c r="H34" s="1">
-        <v>43782.161676834643</v>
       </c>
     </row>
     <row r="35">
@@ -75441,58 +75441,58 @@
         <v>-4009.0753441289712</v>
       </c>
       <c r="D35" s="1">
-        <v>-4009.0753441289712</v>
+        <v>-4009.0753441289771</v>
       </c>
       <c r="E35" s="1">
-        <v>-63565.818181042087</v>
+        <v>-63565.770979082881</v>
       </c>
       <c r="F35" s="1">
         <v>-63565.770979082881</v>
       </c>
       <c r="G35" s="1">
+        <v>43782.161676835007</v>
+      </c>
+      <c r="H35" s="1">
         <v>43782.161676834643</v>
-      </c>
-      <c r="H35" s="1">
-        <v>43782.161676835007</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>24285</v>
+        <v>24286</v>
       </c>
       <c r="B36" t="s">
-        <v>24321</v>
+        <v>24322</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>201604.21968480741</v>
-      </c>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1">
-        <v>337.34758922499998</v>
-      </c>
-      <c r="H36" s="1">
-        <v>253381.7166756459</v>
-      </c>
+        <v>170013.75605207999</v>
+      </c>
+      <c r="F36" s="1">
+        <v>170013.75605207999</v>
+      </c>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24286</v>
+        <v>24285</v>
       </c>
       <c r="B37" t="s">
-        <v>24322</v>
+        <v>24321</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>170013.75605207999</v>
-      </c>
-      <c r="F37" s="1">
-        <v>170013.75605207999</v>
-      </c>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
+        <v>201604.21968480741</v>
+      </c>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1">
+        <v>337.34758922499998</v>
+      </c>
+      <c r="H37" s="1">
+        <v>253381.7166756459</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
@@ -76246,7 +76246,7 @@
         <v>33283.712597372418</v>
       </c>
       <c r="H34" s="1">
-        <v>33283.712597372112</v>
+        <v>33283.712597372418</v>
       </c>
     </row>
     <row r="35">
@@ -76272,7 +76272,7 @@
         <v>33283.712597372112</v>
       </c>
       <c r="H35" s="1">
-        <v>33283.712597372418</v>
+        <v>33283.712597372112</v>
       </c>
     </row>
     <row r="36">
@@ -76297,35 +76297,35 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24284</v>
+        <v>24286</v>
       </c>
       <c r="B37" t="s">
-        <v>24320</v>
+        <v>24322</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>1640.019891895929</v>
-      </c>
-      <c r="F37" s="1"/>
+        <v>207169.67690947151</v>
+      </c>
+      <c r="F37" s="1">
+        <v>207169.67690947151</v>
+      </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24286</v>
+        <v>24284</v>
       </c>
       <c r="B38" t="s">
-        <v>24322</v>
+        <v>24320</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>207169.67690947151</v>
-      </c>
-      <c r="F38" s="1">
-        <v>207169.67690947151</v>
-      </c>
+        <v>1640.019891895929</v>
+      </c>
+      <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
@@ -76913,7 +76913,7 @@
         <v>-47487.012322160823</v>
       </c>
       <c r="F27" s="1">
-        <v>-47487.012322160823</v>
+        <v>-47487.012322160852</v>
       </c>
       <c r="G27" s="1">
         <v>137422.3722114753</v>
@@ -76991,7 +76991,7 @@
         <v>-47487.012322160852</v>
       </c>
       <c r="F31" s="1">
-        <v>-47487.012322160852</v>
+        <v>-47487.012322160823</v>
       </c>
       <c r="G31" s="1">
         <v>137422.3722114753</v>
@@ -77055,7 +77055,7 @@
         <v>-14516.140951382629</v>
       </c>
       <c r="D34" s="1">
-        <v>-14516.15048177604</v>
+        <v>-14516.140951382629</v>
       </c>
       <c r="E34" s="1">
         <v>-63947.039175029808</v>
@@ -77064,7 +77064,7 @@
         <v>-63947.039175030113</v>
       </c>
       <c r="G34" s="1">
-        <v>39248.472782472993</v>
+        <v>39248.472782472847</v>
       </c>
       <c r="H34" s="1">
         <v>39248.472782472847</v>
@@ -77081,7 +77081,7 @@
         <v>-14516.15048177604</v>
       </c>
       <c r="D35" s="1">
-        <v>-14516.140951382629</v>
+        <v>-14516.15048177604</v>
       </c>
       <c r="E35" s="1">
         <v>-63947.039175030113</v>
@@ -77090,7 +77090,7 @@
         <v>-63947.039175029808</v>
       </c>
       <c r="G35" s="1">
-        <v>39248.472782472847</v>
+        <v>39248.472782472993</v>
       </c>
       <c r="H35" s="1">
         <v>39248.472782472993</v>
@@ -77098,55 +77098,55 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>24284</v>
+        <v>24285</v>
       </c>
       <c r="B36" t="s">
-        <v>24320</v>
+        <v>24321</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>1691.532447066628</v>
+        <v>239376.743428952</v>
       </c>
       <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
+      <c r="G36" s="1">
+        <v>402.67289956090139</v>
+      </c>
+      <c r="H36" s="1">
+        <v>298520.24294644757</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24285</v>
+        <v>24286</v>
       </c>
       <c r="B37" t="s">
-        <v>24321</v>
+        <v>24322</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>239376.743428952</v>
-      </c>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1">
-        <v>402.67289956090139</v>
-      </c>
-      <c r="H37" s="1">
-        <v>298520.24294644757</v>
-      </c>
+        <v>200663.39336498949</v>
+      </c>
+      <c r="F37" s="1">
+        <v>200663.39336498949</v>
+      </c>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24286</v>
+        <v>24284</v>
       </c>
       <c r="B38" t="s">
-        <v>24322</v>
+        <v>24320</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>200663.39336498949</v>
-      </c>
-      <c r="F38" s="1">
-        <v>200663.39336498949</v>
-      </c>
+        <v>1691.532447066628</v>
+      </c>
+      <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
@@ -77872,7 +77872,7 @@
         <v>10171.468589380889</v>
       </c>
       <c r="D34" s="1">
-        <v>10171.468589380889</v>
+        <v>10171.459058987501</v>
       </c>
       <c r="E34" s="1">
         <v>-79545.106801385089</v>
@@ -77884,7 +77884,7 @@
         <v>66058.729479423899</v>
       </c>
       <c r="H34" s="1">
-        <v>66058.729479423899</v>
+        <v>66059.10105946564</v>
       </c>
     </row>
     <row r="35">
@@ -77898,7 +77898,7 @@
         <v>10171.459058987501</v>
       </c>
       <c r="D35" s="1">
-        <v>10171.459058987501</v>
+        <v>10171.468589380889</v>
       </c>
       <c r="E35" s="1">
         <v>-79545.106801385089</v>
@@ -77910,60 +77910,60 @@
         <v>66059.10105946564</v>
       </c>
       <c r="H35" s="1">
-        <v>66059.10105946564</v>
+        <v>66058.729479423899</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>24285</v>
+        <v>24286</v>
       </c>
       <c r="B36" t="s">
-        <v>24321</v>
+        <v>24322</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>250754.8245620098</v>
-      </c>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1">
-        <v>442.30808405340002</v>
-      </c>
-      <c r="H36" s="1">
-        <v>313181.58741649322</v>
-      </c>
+        <v>242248.42014405999</v>
+      </c>
+      <c r="F36" s="1">
+        <v>242248.42014405999</v>
+      </c>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24284</v>
+        <v>24285</v>
       </c>
       <c r="B37" t="s">
-        <v>24320</v>
+        <v>24321</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>1625.492093275358</v>
+        <v>250754.8245620098</v>
       </c>
       <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
+      <c r="G37" s="1">
+        <v>442.30808405340002</v>
+      </c>
+      <c r="H37" s="1">
+        <v>313181.58741649322</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>24286</v>
+        <v>24284</v>
       </c>
       <c r="B38" t="s">
-        <v>24322</v>
+        <v>24320</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>242248.42014405999</v>
-      </c>
-      <c r="F38" s="1">
-        <v>242248.42014405999</v>
-      </c>
+        <v>1625.492093275358</v>
+      </c>
+      <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
@@ -78546,7 +78546,7 @@
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1">
-        <v>-25100.989231280721</v>
+        <v>-25100.98923128075</v>
       </c>
       <c r="F27" s="1">
         <v>-25100.98923128075</v>
@@ -78624,7 +78624,7 @@
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1">
-        <v>-25100.98923128075</v>
+        <v>-25100.989231280721</v>
       </c>
       <c r="F31" s="1">
         <v>-25100.989231280721</v>
@@ -78691,7 +78691,7 @@
         <v>63134.524836636163</v>
       </c>
       <c r="D34" s="1">
-        <v>63134.524836636163</v>
+        <v>63134.515306242713</v>
       </c>
       <c r="E34" s="1">
         <v>-60032.164387225363</v>
@@ -78700,7 +78700,7 @@
         <v>-60032.164387225363</v>
       </c>
       <c r="G34" s="1">
-        <v>50492.474199901873</v>
+        <v>50492.474199902237</v>
       </c>
       <c r="H34" s="1">
         <v>50492.474199902237</v>
@@ -78717,7 +78717,7 @@
         <v>63134.515306242713</v>
       </c>
       <c r="D35" s="1">
-        <v>63134.515306242713</v>
+        <v>63134.524836636163</v>
       </c>
       <c r="E35" s="1">
         <v>-60032.164387225363</v>
@@ -78726,7 +78726,7 @@
         <v>-60032.164387225363</v>
       </c>
       <c r="G35" s="1">
-        <v>50492.474199902237</v>
+        <v>50492.474199901873</v>
       </c>
       <c r="H35" s="1">
         <v>50492.474199901873</v>
@@ -78734,39 +78734,39 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>24284</v>
+        <v>24285</v>
       </c>
       <c r="B36" t="s">
-        <v>24320</v>
+        <v>24321</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>1891.473003789004</v>
+        <v>272538.25067318691</v>
       </c>
       <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
+      <c r="G36" s="1">
+        <v>456.40441621169998</v>
+      </c>
+      <c r="H36" s="1">
+        <v>335741.85541967727</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>24285</v>
+        <v>24284</v>
       </c>
       <c r="B37" t="s">
-        <v>24321</v>
+        <v>24320</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>272538.25067318691</v>
+        <v>1891.473003789004</v>
       </c>
       <c r="F37" s="1"/>
-      <c r="G37" s="1">
-        <v>456.40441621169998</v>
-      </c>
-      <c r="H37" s="1">
-        <v>335741.85541967727</v>
-      </c>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">

</xml_diff>